<commit_message>
CI Reports [2026-06-26 06:29]: Login — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report/Feature Reports/Login.xlsx
+++ b/Test Execution Report/Feature Reports/Login.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O21"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="45.83203125" customWidth="1"/>
@@ -464,9 +464,989 @@
         <v>Remarks</v>
       </c>
     </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>TC-LOGIN-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>TC-LOGIN-001 | Valid login redirects to dashboard</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K2" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M2" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N2" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>TC-LOGIN-002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>TC-LOGIN-002 | Login page loads with all required fields</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K3" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M3" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N3" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>TC-LOGIN-003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>TC-LOGIN-003 | Password field is masked by default</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K4" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M4" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N4" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>TC-LOGIN-004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>TC-LOGIN-004 | Password show/hide toggle works</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K5" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M5" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N5" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>TC-LOGIN-005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>TC-LOGIN-005 | Remember Me checkbox toggles correctly</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K6" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M6" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N6" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>TC-LOGIN-006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>TC-LOGIN-006 | Invalid credentials shows error message</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E7" t="str">
+        <v>High</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K7" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M7" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N7" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>TC-LOGIN-007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>TC-LOGIN-007 | Empty username and password blocked</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E8" t="str">
+        <v>High</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G8" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K8" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M8" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N8" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>TC-LOGIN-008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>TC-LOGIN-008 | Valid username with empty password blocked</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E9" t="str">
+        <v>High</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K9" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M9" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N9" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>TC-LOGIN-009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>TC-LOGIN-009 | Empty username with valid password blocked</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E10" t="str">
+        <v>High</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G10" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K10" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M10" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N10" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>TC-LOGIN-010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>TC-LOGIN-010 | Wrong username with correct password rejected</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E11" t="str">
+        <v>High</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K11" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M11" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N11" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>TC-LOGIN-011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>TC-LOGIN-011 | Correct username with wrong password rejected</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E12" t="str">
+        <v>High</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K12" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M12" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N12" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>TC-LOGIN-012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>TC-LOGIN-012 | Username with 256 characters handled gracefully</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K13" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M13" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N13" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>TC-LOGIN-013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>TC-LOGIN-013 | Password with 256 characters handled gracefully</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K14" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M14" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N14" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>TC-LOGIN-014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>TC-LOGIN-014 | Whitespace-only username is rejected</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K15" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M15" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N15" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>TC-LOGIN-015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>TC-LOGIN-015 | Special characters in username handled safely</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G16" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J16" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K16" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M16" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N16" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>TC-LOGIN-016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>TC-LOGIN-016 | SQL injection in username handled safely</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Security</v>
+      </c>
+      <c r="E17" t="str">
+        <v>High</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K17" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M17" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N17" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>TC-LOGIN-017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>TC-LOGIN-017 | SQL injection in password handled safely</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Security</v>
+      </c>
+      <c r="E18" t="str">
+        <v>High</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J18" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K18" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M18" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N18" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>TC-LOGIN-018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>TC-LOGIN-018 | XSS payload in username handled safely</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Security</v>
+      </c>
+      <c r="E19" t="str">
+        <v>High</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K19" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M19" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N19" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>TC-LOGIN-019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>TC-LOGIN-019 | Unauthenticated access redirects to login</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Security</v>
+      </c>
+      <c r="E20" t="str">
+        <v>High</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K20" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L20" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M20" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N20" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>TC-LOGIN-020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>TC-LOGIN-020 | Username login is case-insensitive (behaviour confirmed)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="G21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Perform action
+3. Verify result</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Refer to test-data/loginData.js</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Test should pass per acceptance criteria</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Test passed successfully</v>
+      </c>
+      <c r="K21" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Claude QA Automation</v>
+      </c>
+      <c r="M21" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="N21" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows</v>
+      </c>
+      <c r="O21" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O21"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
CI Reports [2026-06-26 14:22]: Login — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report/Feature Reports/Login.xlsx
+++ b/Test Execution Report/Feature Reports/Login.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P21"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="45.83203125" customWidth="1"/>
@@ -468,9 +468,1009 @@
         <v>Remarks</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>TC-LOGIN-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>TC-LOGIN-001 | Valid login redirects to dashboard</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H2" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I2" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K2" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L2" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N2" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O2" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>TC-LOGIN-002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>TC-LOGIN-002 | Login page loads with all required fields</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H3" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I3" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K3" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L3" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N3" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O3" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TC-LOGIN-003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>TC-LOGIN-003 | Password field is masked by default</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H4" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I4" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K4" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L4" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N4" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O4" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TC-LOGIN-004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>TC-LOGIN-004 | Password show/hide toggle works</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H5" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I5" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K5" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L5" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N5" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O5" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TC-LOGIN-005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>TC-LOGIN-005 | Remember Me checkbox toggles correctly</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H6" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I6" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K6" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L6" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N6" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O6" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TC-LOGIN-006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>TC-LOGIN-006 | Invalid credentials shows error message</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E7" t="str">
+        <v>High</v>
+      </c>
+      <c r="F7" t="str">
+        <v>API</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H7" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I7" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K7" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L7" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N7" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O7" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TC-LOGIN-007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>TC-LOGIN-007 | Empty username and password blocked</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E8" t="str">
+        <v>High</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H8" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I8" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K8" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L8" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N8" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O8" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TC-LOGIN-008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>TC-LOGIN-008 | Valid username with empty password blocked</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E9" t="str">
+        <v>High</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H9" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I9" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K9" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L9" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N9" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O9" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TC-LOGIN-009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>TC-LOGIN-009 | Empty username with valid password blocked</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E10" t="str">
+        <v>High</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H10" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I10" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K10" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L10" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N10" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O10" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TC-LOGIN-010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>TC-LOGIN-010 | Wrong username with correct password rejected</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E11" t="str">
+        <v>High</v>
+      </c>
+      <c r="F11" t="str">
+        <v>API</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H11" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I11" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K11" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L11" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N11" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O11" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TC-LOGIN-011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>TC-LOGIN-011 | Correct username with wrong password rejected</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E12" t="str">
+        <v>High</v>
+      </c>
+      <c r="F12" t="str">
+        <v>API</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H12" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I12" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K12" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L12" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N12" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O12" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TC-LOGIN-012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>TC-LOGIN-012 | Username with 256 characters handled gracefully</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="F13" t="str">
+        <v>API</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H13" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I13" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K13" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L13" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N13" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O13" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TC-LOGIN-013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>TC-LOGIN-013 | Password with 256 characters handled gracefully</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="F14" t="str">
+        <v>API</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H14" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I14" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K14" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L14" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M14" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N14" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O14" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TC-LOGIN-014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>TC-LOGIN-014 | Whitespace-only username is rejected</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H15" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I15" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K15" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L15" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M15" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N15" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O15" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TC-LOGIN-015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>TC-LOGIN-015 | Special characters in username handled safely</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="F16" t="str">
+        <v>API</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H16" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I16" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J16" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K16" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L16" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M16" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N16" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O16" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TC-LOGIN-016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>TC-LOGIN-016 | SQL injection in username handled safely</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Security</v>
+      </c>
+      <c r="E17" t="str">
+        <v>High</v>
+      </c>
+      <c r="F17" t="str">
+        <v>API</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H17" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I17" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K17" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L17" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M17" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N17" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O17" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TC-LOGIN-017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>TC-LOGIN-017 | SQL injection in password handled safely</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Security</v>
+      </c>
+      <c r="E18" t="str">
+        <v>High</v>
+      </c>
+      <c r="F18" t="str">
+        <v>API</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H18" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I18" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J18" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K18" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L18" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M18" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N18" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O18" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TC-LOGIN-018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>TC-LOGIN-018 | XSS payload in username handled safely</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Security</v>
+      </c>
+      <c r="E19" t="str">
+        <v>High</v>
+      </c>
+      <c r="F19" t="str">
+        <v>API</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H19" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I19" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K19" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L19" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M19" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N19" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O19" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TC-LOGIN-019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>TC-LOGIN-019 | Unauthenticated access redirects to login</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Security</v>
+      </c>
+      <c r="E20" t="str">
+        <v>High</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H20" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I20" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K20" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L20" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M20" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N20" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O20" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TC-LOGIN-020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>TC-LOGIN-020 | Username login is case-insensitive (behaviour confirmed)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Login</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F21" t="str">
+        <v>API</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
+      </c>
+      <c r="H21" t="str">
+        <v>(See Playwright spec: tests/login.spec.js)</v>
+      </c>
+      <c r="I21" t="str">
+        <v>See test-data/loginData.js</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Test assertions pass per spec definition</v>
+      </c>
+      <c r="K21" t="str">
+        <v>All assertions passed via Playwright</v>
+      </c>
+      <c r="L21" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="M21" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="N21" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="O21" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="P21" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P21"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>